<commit_message>
Complete FastAPI backend with analytics pipeline
</commit_message>
<xml_diff>
--- a/backend/data/exports/reports/output/business_insights.xlsx
+++ b/backend/data/exports/reports/output/business_insights.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RTE-9810A785</t>
+          <t>RTE-7F91720C</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[{"Metric": "Average Delay Hours", "Value": 7.290870044052863}, {"Metric": "Temperature Compliance Rate (%)", "Value": 89.97797356828194}, {"Metric": "Humidity Compliance Rate (%)", "Value": 93.5022026431718}, {"Metric": "Battery Health Rate (%)", "Value": 91.96035242290749}, {"Metric": "Delay Compliance Rate (%)", "Value": 60.352422907488986}, {"Metric": "Most Delayed Route", "Value": "RTE-9810A785"}]</t>
+          <t>[{"Metric": "Average Delay Hours", "Value": 7.290870044052863}, {"Metric": "Temperature Compliance Rate (%)", "Value": 89.97797356828194}, {"Metric": "Humidity Compliance Rate (%)", "Value": 93.5022026431718}, {"Metric": "Battery Health Rate (%)", "Value": 91.96035242290749}, {"Metric": "Delay Compliance Rate (%)", "Value": 60.352422907488986}, {"Metric": "Most Delayed Route", "Value": "RTE-7F91720C"}]</t>
         </is>
       </c>
     </row>

</xml_diff>